<commit_message>
UK daily ratings for 2026-05-06
</commit_message>
<xml_diff>
--- a/output/daily_ratings/uk_ratings_2026-05-06.xlsx
+++ b/output/daily_ratings/uk_ratings_2026-05-06.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P70"/>
+  <dimension ref="A1:P148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2544,17 +2544,17 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Saffron Dandy (IRE)</t>
+          <t>Silent Strike (IRE)</t>
         </is>
       </c>
       <c r="I36" t="n">
         <v>3</v>
       </c>
       <c r="J36" t="n">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="K36" t="n">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="n">
@@ -2600,17 +2600,17 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Silent Strike (IRE)</t>
+          <t>Saffron Dandy (IRE)</t>
         </is>
       </c>
       <c r="I37" t="n">
         <v>3</v>
       </c>
       <c r="J37" t="n">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="K37" t="n">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="n">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Norman Invasion</t>
+          <t>Alfaraz</t>
         </is>
       </c>
       <c r="I50" t="n">
@@ -3384,7 +3384,7 @@
         <v>133</v>
       </c>
       <c r="K50" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="n">
@@ -3430,7 +3430,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Alfaraz</t>
+          <t>Norman Invasion</t>
         </is>
       </c>
       <c r="I51" t="n">
@@ -3440,7 +3440,7 @@
         <v>133</v>
       </c>
       <c r="K51" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="n">
@@ -4587,6 +4587,4660 @@
       <c r="P70" t="n">
         <v>0</v>
       </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" t="n">
+        <v>8</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>6</v>
+      </c>
+      <c r="G71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Sceptic (IRE)</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>6</v>
+      </c>
+      <c r="J71" t="n">
+        <v>135</v>
+      </c>
+      <c r="K71" t="n">
+        <v>56</v>
+      </c>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="N71" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P71" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>1</v>
+      </c>
+      <c r="C72" t="n">
+        <v>8</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>6</v>
+      </c>
+      <c r="G72" t="n">
+        <v>2</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Berning Hot (IRE)</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>4</v>
+      </c>
+      <c r="J72" t="n">
+        <v>135</v>
+      </c>
+      <c r="K72" t="n">
+        <v>56</v>
+      </c>
+      <c r="L72" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M72" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="N72" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P72" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>1</v>
+      </c>
+      <c r="C73" t="n">
+        <v>8</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>6</v>
+      </c>
+      <c r="G73" t="n">
+        <v>3</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Miss Chester (IRE)</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>4</v>
+      </c>
+      <c r="J73" t="n">
+        <v>131</v>
+      </c>
+      <c r="K73" t="n">
+        <v>52</v>
+      </c>
+      <c r="L73" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="M73" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="N73" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P73" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>1</v>
+      </c>
+      <c r="C74" t="n">
+        <v>8</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>6</v>
+      </c>
+      <c r="G74" t="n">
+        <v>4</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Aim For The Bull (IRE)</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>4</v>
+      </c>
+      <c r="J74" t="n">
+        <v>133</v>
+      </c>
+      <c r="K74" t="n">
+        <v>54</v>
+      </c>
+      <c r="L74" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="M74" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="N74" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P74" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>1</v>
+      </c>
+      <c r="C75" t="n">
+        <v>8</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>6</v>
+      </c>
+      <c r="G75" t="n">
+        <v>5</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>King Of Speed (IRE)</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>7</v>
+      </c>
+      <c r="J75" t="n">
+        <v>135</v>
+      </c>
+      <c r="K75" t="n">
+        <v>56</v>
+      </c>
+      <c r="L75" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="M75" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="N75" t="n">
+        <v>36</v>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P75" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>1</v>
+      </c>
+      <c r="C76" t="n">
+        <v>8</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>6</v>
+      </c>
+      <c r="G76" t="n">
+        <v>6</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Dinah Myte</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>4</v>
+      </c>
+      <c r="J76" t="n">
+        <v>126</v>
+      </c>
+      <c r="K76" t="n">
+        <v>47</v>
+      </c>
+      <c r="L76" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="M76" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="N76" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P76" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1</v>
+      </c>
+      <c r="C77" t="n">
+        <v>8</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>6</v>
+      </c>
+      <c r="G77" t="n">
+        <v>7</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Port Noir</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>9</v>
+      </c>
+      <c r="J77" t="n">
+        <v>135</v>
+      </c>
+      <c r="K77" t="n">
+        <v>56</v>
+      </c>
+      <c r="L77" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="M77" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="N77" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P77" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" t="n">
+        <v>8</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>6</v>
+      </c>
+      <c r="G78" t="n">
+        <v>8</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Marchetti (IRE)</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>9</v>
+      </c>
+      <c r="J78" t="n">
+        <v>124</v>
+      </c>
+      <c r="K78" t="n">
+        <v>45</v>
+      </c>
+      <c r="L78" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="M78" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="N78" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P78" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>1</v>
+      </c>
+      <c r="C79" t="n">
+        <v>8</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>6</v>
+      </c>
+      <c r="G79" t="n">
+        <v>9</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Daddy Chill (IRE)</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>4</v>
+      </c>
+      <c r="J79" t="n">
+        <v>129</v>
+      </c>
+      <c r="K79" t="n">
+        <v>50</v>
+      </c>
+      <c r="L79" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="M79" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="N79" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P79" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>2</v>
+      </c>
+      <c r="C80" t="n">
+        <v>8</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>5</v>
+      </c>
+      <c r="G80" t="n">
+        <v>1</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Blues And Royals (IRE)</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>3</v>
+      </c>
+      <c r="J80" t="n">
+        <v>135</v>
+      </c>
+      <c r="K80" t="n">
+        <v>75</v>
+      </c>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="n">
+        <v>99.19</v>
+      </c>
+      <c r="N80" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P80" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>2</v>
+      </c>
+      <c r="C81" t="n">
+        <v>8</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>5</v>
+      </c>
+      <c r="G81" t="n">
+        <v>2</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Victory Ace</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>3</v>
+      </c>
+      <c r="J81" t="n">
+        <v>133</v>
+      </c>
+      <c r="K81" t="n">
+        <v>73</v>
+      </c>
+      <c r="L81" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="M81" t="n">
+        <v>99.19</v>
+      </c>
+      <c r="N81" t="n">
+        <v>71.09999999999999</v>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P81" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>2</v>
+      </c>
+      <c r="C82" t="n">
+        <v>8</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>5</v>
+      </c>
+      <c r="G82" t="n">
+        <v>3</v>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Trio</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>3</v>
+      </c>
+      <c r="J82" t="n">
+        <v>131</v>
+      </c>
+      <c r="K82" t="n">
+        <v>71</v>
+      </c>
+      <c r="L82" t="n">
+        <v>2</v>
+      </c>
+      <c r="M82" t="n">
+        <v>99.19</v>
+      </c>
+      <c r="N82" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P82" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>2</v>
+      </c>
+      <c r="C83" t="n">
+        <v>8</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>5</v>
+      </c>
+      <c r="G83" t="n">
+        <v>4</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Booziebrunch (IRE)</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>3</v>
+      </c>
+      <c r="J83" t="n">
+        <v>132</v>
+      </c>
+      <c r="K83" t="n">
+        <v>72</v>
+      </c>
+      <c r="L83" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="M83" t="n">
+        <v>99.19</v>
+      </c>
+      <c r="N83" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P83" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>2</v>
+      </c>
+      <c r="C84" t="n">
+        <v>8</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>5</v>
+      </c>
+      <c r="G84" t="n">
+        <v>5</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Melody De Vega (IRE)</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>3</v>
+      </c>
+      <c r="J84" t="n">
+        <v>134</v>
+      </c>
+      <c r="K84" t="n">
+        <v>74</v>
+      </c>
+      <c r="L84" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="M84" t="n">
+        <v>99.19</v>
+      </c>
+      <c r="N84" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P84" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>2</v>
+      </c>
+      <c r="C85" t="n">
+        <v>8</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>5</v>
+      </c>
+      <c r="G85" t="n">
+        <v>6</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>High Approval (IRE)</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>3</v>
+      </c>
+      <c r="J85" t="n">
+        <v>135</v>
+      </c>
+      <c r="K85" t="n">
+        <v>75</v>
+      </c>
+      <c r="L85" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="M85" t="n">
+        <v>99.19</v>
+      </c>
+      <c r="N85" t="n">
+        <v>63.9</v>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>2</v>
+      </c>
+      <c r="C86" t="n">
+        <v>8</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>5</v>
+      </c>
+      <c r="G86" t="n">
+        <v>7</v>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Bennyworth (IRE)</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>3</v>
+      </c>
+      <c r="J86" t="n">
+        <v>125</v>
+      </c>
+      <c r="K86" t="n">
+        <v>65</v>
+      </c>
+      <c r="L86" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="M86" t="n">
+        <v>99.19</v>
+      </c>
+      <c r="N86" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P86" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>2</v>
+      </c>
+      <c r="C87" t="n">
+        <v>8</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>5</v>
+      </c>
+      <c r="G87" t="n">
+        <v>8</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Chapmans Peak</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>3</v>
+      </c>
+      <c r="J87" t="n">
+        <v>132</v>
+      </c>
+      <c r="K87" t="n">
+        <v>72</v>
+      </c>
+      <c r="L87" t="n">
+        <v>8.550000000000001</v>
+      </c>
+      <c r="M87" t="n">
+        <v>99.19</v>
+      </c>
+      <c r="N87" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P87" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>2</v>
+      </c>
+      <c r="C88" t="n">
+        <v>8</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>5</v>
+      </c>
+      <c r="G88" t="n">
+        <v>9</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Crafty Blue (IRE)</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>3</v>
+      </c>
+      <c r="J88" t="n">
+        <v>133</v>
+      </c>
+      <c r="K88" t="n">
+        <v>73</v>
+      </c>
+      <c r="L88" t="n">
+        <v>56.55</v>
+      </c>
+      <c r="M88" t="n">
+        <v>99.19</v>
+      </c>
+      <c r="N88" t="n">
+        <v>-33.8</v>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P88" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>3</v>
+      </c>
+      <c r="C89" t="n">
+        <v>10.99545454545455</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>4</v>
+      </c>
+      <c r="G89" t="n">
+        <v>1</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Brilliant Star</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>3</v>
+      </c>
+      <c r="J89" t="n">
+        <v>132</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="n">
+        <v>140.64</v>
+      </c>
+      <c r="N89" t="n">
+        <v>69.09999999999999</v>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P89" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>3</v>
+      </c>
+      <c r="C90" t="n">
+        <v>10.99545454545455</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>4</v>
+      </c>
+      <c r="G90" t="n">
+        <v>2</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Eloquencia</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>3</v>
+      </c>
+      <c r="J90" t="n">
+        <v>125</v>
+      </c>
+      <c r="K90" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="M90" t="n">
+        <v>140.64</v>
+      </c>
+      <c r="N90" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P90" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>3</v>
+      </c>
+      <c r="C91" t="n">
+        <v>10.99545454545455</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>4</v>
+      </c>
+      <c r="G91" t="n">
+        <v>3</v>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Golden Step</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>3</v>
+      </c>
+      <c r="J91" t="n">
+        <v>123</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" t="n">
+        <v>13</v>
+      </c>
+      <c r="M91" t="n">
+        <v>140.64</v>
+      </c>
+      <c r="N91" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P91" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>3</v>
+      </c>
+      <c r="C92" t="n">
+        <v>10.99545454545455</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>4</v>
+      </c>
+      <c r="G92" t="n">
+        <v>4</v>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Shirakawa</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>3</v>
+      </c>
+      <c r="J92" t="n">
+        <v>125</v>
+      </c>
+      <c r="K92" t="n">
+        <v>0</v>
+      </c>
+      <c r="L92" t="n">
+        <v>15</v>
+      </c>
+      <c r="M92" t="n">
+        <v>140.64</v>
+      </c>
+      <c r="N92" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P92" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>3</v>
+      </c>
+      <c r="C93" t="n">
+        <v>10.99545454545455</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>4</v>
+      </c>
+      <c r="G93" t="n">
+        <v>5</v>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Dream Of Ithaca</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>3</v>
+      </c>
+      <c r="J93" t="n">
+        <v>123</v>
+      </c>
+      <c r="K93" t="n">
+        <v>49</v>
+      </c>
+      <c r="L93" t="n">
+        <v>19</v>
+      </c>
+      <c r="M93" t="n">
+        <v>140.64</v>
+      </c>
+      <c r="N93" t="n">
+        <v>22</v>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P93" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>3</v>
+      </c>
+      <c r="C94" t="n">
+        <v>10.99545454545455</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>4</v>
+      </c>
+      <c r="G94" t="n">
+        <v>6</v>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Joanna Hiffernan</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>4</v>
+      </c>
+      <c r="J94" t="n">
+        <v>142</v>
+      </c>
+      <c r="K94" t="n">
+        <v>0</v>
+      </c>
+      <c r="L94" t="n">
+        <v>21.25</v>
+      </c>
+      <c r="M94" t="n">
+        <v>140.64</v>
+      </c>
+      <c r="N94" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P94" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>3</v>
+      </c>
+      <c r="C95" t="n">
+        <v>10.99545454545455</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>4</v>
+      </c>
+      <c r="G95" t="n">
+        <v>7</v>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Emerald Reine</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>3</v>
+      </c>
+      <c r="J95" t="n">
+        <v>121</v>
+      </c>
+      <c r="K95" t="n">
+        <v>0</v>
+      </c>
+      <c r="L95" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="M95" t="n">
+        <v>140.64</v>
+      </c>
+      <c r="N95" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P95" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>3</v>
+      </c>
+      <c r="C96" t="n">
+        <v>10.99545454545455</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>4</v>
+      </c>
+      <c r="G96" t="n">
+        <v>8</v>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Blue Birdie (IRE)</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>3</v>
+      </c>
+      <c r="J96" t="n">
+        <v>121</v>
+      </c>
+      <c r="K96" t="n">
+        <v>0</v>
+      </c>
+      <c r="L96" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="M96" t="n">
+        <v>140.64</v>
+      </c>
+      <c r="N96" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P96" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>4</v>
+      </c>
+      <c r="C97" t="n">
+        <v>7</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>5</v>
+      </c>
+      <c r="G97" t="n">
+        <v>1</v>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Venetian Gold (IRE)</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>3</v>
+      </c>
+      <c r="J97" t="n">
+        <v>128</v>
+      </c>
+      <c r="K97" t="n">
+        <v>0</v>
+      </c>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="N97" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P97" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>4</v>
+      </c>
+      <c r="C98" t="n">
+        <v>7</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>5</v>
+      </c>
+      <c r="G98" t="n">
+        <v>2</v>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Perdy In Paris</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>3</v>
+      </c>
+      <c r="J98" t="n">
+        <v>126</v>
+      </c>
+      <c r="K98" t="n">
+        <v>0</v>
+      </c>
+      <c r="L98" t="n">
+        <v>1</v>
+      </c>
+      <c r="M98" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="N98" t="n">
+        <v>63.9</v>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P98" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>4</v>
+      </c>
+      <c r="C99" t="n">
+        <v>7</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>5</v>
+      </c>
+      <c r="G99" t="n">
+        <v>3</v>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Cixi (USA)</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>3</v>
+      </c>
+      <c r="J99" t="n">
+        <v>128</v>
+      </c>
+      <c r="K99" t="n">
+        <v>75</v>
+      </c>
+      <c r="L99" t="n">
+        <v>2</v>
+      </c>
+      <c r="M99" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="N99" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P99" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>4</v>
+      </c>
+      <c r="C100" t="n">
+        <v>7</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>5</v>
+      </c>
+      <c r="G100" t="n">
+        <v>4</v>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Iqbaal (IRE)</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>3</v>
+      </c>
+      <c r="J100" t="n">
+        <v>124</v>
+      </c>
+      <c r="K100" t="n">
+        <v>0</v>
+      </c>
+      <c r="L100" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="M100" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="N100" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P100" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>4</v>
+      </c>
+      <c r="C101" t="n">
+        <v>7</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>5</v>
+      </c>
+      <c r="G101" t="n">
+        <v>5</v>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Coxys Star</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>3</v>
+      </c>
+      <c r="J101" t="n">
+        <v>124</v>
+      </c>
+      <c r="K101" t="n">
+        <v>0</v>
+      </c>
+      <c r="L101" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="M101" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="N101" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P101" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>4</v>
+      </c>
+      <c r="C102" t="n">
+        <v>7</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>5</v>
+      </c>
+      <c r="G102" t="n">
+        <v>6</v>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Komodo Rose</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>3</v>
+      </c>
+      <c r="J102" t="n">
+        <v>126</v>
+      </c>
+      <c r="K102" t="n">
+        <v>0</v>
+      </c>
+      <c r="L102" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="M102" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="N102" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P102" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>4</v>
+      </c>
+      <c r="C103" t="n">
+        <v>7</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>5</v>
+      </c>
+      <c r="G103" t="n">
+        <v>7</v>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Elshie (IRE)</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>3</v>
+      </c>
+      <c r="J103" t="n">
+        <v>128</v>
+      </c>
+      <c r="K103" t="n">
+        <v>0</v>
+      </c>
+      <c r="L103" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="M103" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="N103" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P103" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>4</v>
+      </c>
+      <c r="C104" t="n">
+        <v>7</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>5</v>
+      </c>
+      <c r="G104" t="n">
+        <v>8</v>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Starborn (IRE)</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>3</v>
+      </c>
+      <c r="J104" t="n">
+        <v>128</v>
+      </c>
+      <c r="K104" t="n">
+        <v>0</v>
+      </c>
+      <c r="L104" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="M104" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="N104" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P104" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>4</v>
+      </c>
+      <c r="C105" t="n">
+        <v>7</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>5</v>
+      </c>
+      <c r="G105" t="n">
+        <v>9</v>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Sierra Sue (IRE)</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>3</v>
+      </c>
+      <c r="J105" t="n">
+        <v>128</v>
+      </c>
+      <c r="K105" t="n">
+        <v>0</v>
+      </c>
+      <c r="L105" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="M105" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="N105" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P105" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>4</v>
+      </c>
+      <c r="C106" t="n">
+        <v>7</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>5</v>
+      </c>
+      <c r="G106" t="n">
+        <v>10</v>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Sterling Fortune</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>3</v>
+      </c>
+      <c r="J106" t="n">
+        <v>128</v>
+      </c>
+      <c r="K106" t="n">
+        <v>0</v>
+      </c>
+      <c r="L106" t="n">
+        <v>9.050000000000001</v>
+      </c>
+      <c r="M106" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="N106" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P106" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>4</v>
+      </c>
+      <c r="C107" t="n">
+        <v>7</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>5</v>
+      </c>
+      <c r="G107" t="n">
+        <v>11</v>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Ronstadt</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>3</v>
+      </c>
+      <c r="J107" t="n">
+        <v>128</v>
+      </c>
+      <c r="K107" t="n">
+        <v>0</v>
+      </c>
+      <c r="L107" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="M107" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="N107" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P107" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>4</v>
+      </c>
+      <c r="C108" t="n">
+        <v>7</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>5</v>
+      </c>
+      <c r="G108" t="n">
+        <v>12</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Katies Song</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>3</v>
+      </c>
+      <c r="J108" t="n">
+        <v>128</v>
+      </c>
+      <c r="K108" t="n">
+        <v>0</v>
+      </c>
+      <c r="L108" t="n">
+        <v>9.85</v>
+      </c>
+      <c r="M108" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="N108" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P108" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>4</v>
+      </c>
+      <c r="C109" t="n">
+        <v>7</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>5</v>
+      </c>
+      <c r="G109" t="n">
+        <v>13</v>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Lady Of Chivalry (IRE)</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>4</v>
+      </c>
+      <c r="J109" t="n">
+        <v>138</v>
+      </c>
+      <c r="K109" t="n">
+        <v>0</v>
+      </c>
+      <c r="L109" t="n">
+        <v>12.35</v>
+      </c>
+      <c r="M109" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="N109" t="n">
+        <v>32</v>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P109" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>4</v>
+      </c>
+      <c r="C110" t="n">
+        <v>7</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>5</v>
+      </c>
+      <c r="G110" t="n">
+        <v>14</v>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Snow Day</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>3</v>
+      </c>
+      <c r="J110" t="n">
+        <v>124</v>
+      </c>
+      <c r="K110" t="n">
+        <v>0</v>
+      </c>
+      <c r="L110" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="M110" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="N110" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P110" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>5</v>
+      </c>
+      <c r="C111" t="n">
+        <v>7</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>4</v>
+      </c>
+      <c r="G111" t="n">
+        <v>1</v>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Im Workin On It</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>4</v>
+      </c>
+      <c r="J111" t="n">
+        <v>136</v>
+      </c>
+      <c r="K111" t="n">
+        <v>81</v>
+      </c>
+      <c r="L111" t="inlineStr"/>
+      <c r="M111" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="N111" t="n">
+        <v>75</v>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P111" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>5</v>
+      </c>
+      <c r="C112" t="n">
+        <v>7</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>4</v>
+      </c>
+      <c r="G112" t="n">
+        <v>2</v>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Kit Gabriel (IRE)</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>7</v>
+      </c>
+      <c r="J112" t="n">
+        <v>123</v>
+      </c>
+      <c r="K112" t="n">
+        <v>68</v>
+      </c>
+      <c r="L112" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M112" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="N112" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P112" t="n">
+        <v>-3.5</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>5</v>
+      </c>
+      <c r="C113" t="n">
+        <v>7</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>4</v>
+      </c>
+      <c r="G113" t="n">
+        <v>3</v>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Blue Prince (IRE)</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>5</v>
+      </c>
+      <c r="J113" t="n">
+        <v>133</v>
+      </c>
+      <c r="K113" t="n">
+        <v>78</v>
+      </c>
+      <c r="L113" t="n">
+        <v>1</v>
+      </c>
+      <c r="M113" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="N113" t="n">
+        <v>71</v>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P113" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>5</v>
+      </c>
+      <c r="C114" t="n">
+        <v>7</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>4</v>
+      </c>
+      <c r="G114" t="n">
+        <v>4</v>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Prosperitas (IRE)</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>4</v>
+      </c>
+      <c r="J114" t="n">
+        <v>137</v>
+      </c>
+      <c r="K114" t="n">
+        <v>82</v>
+      </c>
+      <c r="L114" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="M114" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="N114" t="n">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P114" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>5</v>
+      </c>
+      <c r="C115" t="n">
+        <v>7</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>4</v>
+      </c>
+      <c r="G115" t="n">
+        <v>5</v>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Tea Sea (FR)</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>6</v>
+      </c>
+      <c r="J115" t="n">
+        <v>126</v>
+      </c>
+      <c r="K115" t="n">
+        <v>71</v>
+      </c>
+      <c r="L115" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="M115" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="N115" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P115" t="n">
+        <v>-4</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>5</v>
+      </c>
+      <c r="C116" t="n">
+        <v>7</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>4</v>
+      </c>
+      <c r="G116" t="n">
+        <v>6</v>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Farasi Lane (IRE)</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>8</v>
+      </c>
+      <c r="J116" t="n">
+        <v>136</v>
+      </c>
+      <c r="K116" t="n">
+        <v>81</v>
+      </c>
+      <c r="L116" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="M116" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="N116" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P116" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>5</v>
+      </c>
+      <c r="C117" t="n">
+        <v>7</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>4</v>
+      </c>
+      <c r="G117" t="n">
+        <v>7</v>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Arctician (IRE)</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>8</v>
+      </c>
+      <c r="J117" t="n">
+        <v>133</v>
+      </c>
+      <c r="K117" t="n">
+        <v>78</v>
+      </c>
+      <c r="L117" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="M117" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="N117" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P117" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>5</v>
+      </c>
+      <c r="C118" t="n">
+        <v>7</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>4</v>
+      </c>
+      <c r="G118" t="n">
+        <v>8</v>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Mr Baloo (IRE)</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>5</v>
+      </c>
+      <c r="J118" t="n">
+        <v>136</v>
+      </c>
+      <c r="K118" t="n">
+        <v>81</v>
+      </c>
+      <c r="L118" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="M118" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="N118" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P118" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>5</v>
+      </c>
+      <c r="C119" t="n">
+        <v>7</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>4</v>
+      </c>
+      <c r="G119" t="n">
+        <v>9</v>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Ribenska (IRE)</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>4</v>
+      </c>
+      <c r="J119" t="n">
+        <v>128</v>
+      </c>
+      <c r="K119" t="n">
+        <v>73</v>
+      </c>
+      <c r="L119" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="M119" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="N119" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P119" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>5</v>
+      </c>
+      <c r="C120" t="n">
+        <v>7</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>4</v>
+      </c>
+      <c r="G120" t="n">
+        <v>10</v>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Notimeforchitchat (IRE)</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>4</v>
+      </c>
+      <c r="J120" t="n">
+        <v>133</v>
+      </c>
+      <c r="K120" t="n">
+        <v>78</v>
+      </c>
+      <c r="L120" t="n">
+        <v>5.98</v>
+      </c>
+      <c r="M120" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="N120" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P120" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>5</v>
+      </c>
+      <c r="C121" t="n">
+        <v>7</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>4</v>
+      </c>
+      <c r="G121" t="n">
+        <v>11</v>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Iconic Times</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>4</v>
+      </c>
+      <c r="J121" t="n">
+        <v>121</v>
+      </c>
+      <c r="K121" t="n">
+        <v>66</v>
+      </c>
+      <c r="L121" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="M121" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="N121" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P121" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>5</v>
+      </c>
+      <c r="C122" t="n">
+        <v>7</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>4</v>
+      </c>
+      <c r="G122" t="n">
+        <v>12</v>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Receipt</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>4</v>
+      </c>
+      <c r="J122" t="n">
+        <v>128</v>
+      </c>
+      <c r="K122" t="n">
+        <v>73</v>
+      </c>
+      <c r="L122" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="M122" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="N122" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P122" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>5</v>
+      </c>
+      <c r="C123" t="n">
+        <v>7</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>4</v>
+      </c>
+      <c r="G123" t="n">
+        <v>13</v>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Zero Carbon (FR)</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>7</v>
+      </c>
+      <c r="J123" t="n">
+        <v>127</v>
+      </c>
+      <c r="K123" t="n">
+        <v>72</v>
+      </c>
+      <c r="L123" t="n">
+        <v>7.68</v>
+      </c>
+      <c r="M123" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="N123" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P123" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>5</v>
+      </c>
+      <c r="C124" t="n">
+        <v>7</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>4</v>
+      </c>
+      <c r="G124" t="n">
+        <v>14</v>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Silca Bay</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>4</v>
+      </c>
+      <c r="J124" t="n">
+        <v>131</v>
+      </c>
+      <c r="K124" t="n">
+        <v>76</v>
+      </c>
+      <c r="L124" t="n">
+        <v>41.68</v>
+      </c>
+      <c r="M124" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="N124" t="n">
+        <v>-23.7</v>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P124" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>6</v>
+      </c>
+      <c r="C125" t="n">
+        <v>7</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>6</v>
+      </c>
+      <c r="G125" t="n">
+        <v>1</v>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Yehudi (IRE)</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>4</v>
+      </c>
+      <c r="J125" t="n">
+        <v>128</v>
+      </c>
+      <c r="K125" t="n">
+        <v>58</v>
+      </c>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="N125" t="n">
+        <v>65</v>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P125" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>6</v>
+      </c>
+      <c r="C126" t="n">
+        <v>7</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>6</v>
+      </c>
+      <c r="G126" t="n">
+        <v>2</v>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Bint Havana Gold</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>5</v>
+      </c>
+      <c r="J126" t="n">
+        <v>134</v>
+      </c>
+      <c r="K126" t="n">
+        <v>64</v>
+      </c>
+      <c r="L126" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="M126" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="N126" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P126" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>6</v>
+      </c>
+      <c r="C127" t="n">
+        <v>7</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>6</v>
+      </c>
+      <c r="G127" t="n">
+        <v>3</v>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Monsieur Patat</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>9</v>
+      </c>
+      <c r="J127" t="n">
+        <v>135</v>
+      </c>
+      <c r="K127" t="n">
+        <v>65</v>
+      </c>
+      <c r="L127" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="M127" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="N127" t="n">
+        <v>61</v>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P127" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>6</v>
+      </c>
+      <c r="C128" t="n">
+        <v>7</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>6</v>
+      </c>
+      <c r="G128" t="n">
+        <v>4</v>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Divine Wish</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>4</v>
+      </c>
+      <c r="J128" t="n">
+        <v>134</v>
+      </c>
+      <c r="K128" t="n">
+        <v>64</v>
+      </c>
+      <c r="L128" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="M128" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="N128" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P128" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>6</v>
+      </c>
+      <c r="C129" t="n">
+        <v>7</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>6</v>
+      </c>
+      <c r="G129" t="n">
+        <v>5</v>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Ajrad</t>
+        </is>
+      </c>
+      <c r="I129" t="n">
+        <v>8</v>
+      </c>
+      <c r="J129" t="n">
+        <v>129</v>
+      </c>
+      <c r="K129" t="n">
+        <v>59</v>
+      </c>
+      <c r="L129" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="M129" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="N129" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P129" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>6</v>
+      </c>
+      <c r="C130" t="n">
+        <v>7</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>6</v>
+      </c>
+      <c r="G130" t="n">
+        <v>6</v>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Future Cutlet (IRE)</t>
+        </is>
+      </c>
+      <c r="I130" t="n">
+        <v>5</v>
+      </c>
+      <c r="J130" t="n">
+        <v>129</v>
+      </c>
+      <c r="K130" t="n">
+        <v>59</v>
+      </c>
+      <c r="L130" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="M130" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="N130" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P130" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>6</v>
+      </c>
+      <c r="C131" t="n">
+        <v>7</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>6</v>
+      </c>
+      <c r="G131" t="n">
+        <v>7</v>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Luminous Warrior (IRE)</t>
+        </is>
+      </c>
+      <c r="I131" t="n">
+        <v>4</v>
+      </c>
+      <c r="J131" t="n">
+        <v>133</v>
+      </c>
+      <c r="K131" t="n">
+        <v>63</v>
+      </c>
+      <c r="L131" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="M131" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="N131" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P131" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>6</v>
+      </c>
+      <c r="C132" t="n">
+        <v>7</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F132" t="n">
+        <v>6</v>
+      </c>
+      <c r="G132" t="n">
+        <v>8</v>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Orbital Chime</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>6</v>
+      </c>
+      <c r="J132" t="n">
+        <v>131</v>
+      </c>
+      <c r="K132" t="n">
+        <v>61</v>
+      </c>
+      <c r="L132" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="M132" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="N132" t="n">
+        <v>51</v>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P132" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>6</v>
+      </c>
+      <c r="C133" t="n">
+        <v>7</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>6</v>
+      </c>
+      <c r="G133" t="n">
+        <v>9</v>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Taskheer (IRE)</t>
+        </is>
+      </c>
+      <c r="I133" t="n">
+        <v>8</v>
+      </c>
+      <c r="J133" t="n">
+        <v>119</v>
+      </c>
+      <c r="K133" t="n">
+        <v>49</v>
+      </c>
+      <c r="L133" t="n">
+        <v>8</v>
+      </c>
+      <c r="M133" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="N133" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P133" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>6</v>
+      </c>
+      <c r="C134" t="n">
+        <v>7</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F134" t="n">
+        <v>6</v>
+      </c>
+      <c r="G134" t="n">
+        <v>10</v>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Withoutfurtherado (IRE)</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>4</v>
+      </c>
+      <c r="J134" t="n">
+        <v>132</v>
+      </c>
+      <c r="K134" t="n">
+        <v>62</v>
+      </c>
+      <c r="L134" t="n">
+        <v>10</v>
+      </c>
+      <c r="M134" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="N134" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P134" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>6</v>
+      </c>
+      <c r="C135" t="n">
+        <v>7</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F135" t="n">
+        <v>6</v>
+      </c>
+      <c r="G135" t="n">
+        <v>11</v>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Bonnita</t>
+        </is>
+      </c>
+      <c r="I135" t="n">
+        <v>4</v>
+      </c>
+      <c r="J135" t="n">
+        <v>130</v>
+      </c>
+      <c r="K135" t="n">
+        <v>60</v>
+      </c>
+      <c r="L135" t="n">
+        <v>19</v>
+      </c>
+      <c r="M135" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="N135" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P135" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>6</v>
+      </c>
+      <c r="C136" t="n">
+        <v>7</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F136" t="n">
+        <v>6</v>
+      </c>
+      <c r="G136" t="n">
+        <v>12</v>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Noble Phoenix (IRE)</t>
+        </is>
+      </c>
+      <c r="I136" t="n">
+        <v>4</v>
+      </c>
+      <c r="J136" t="n">
+        <v>116</v>
+      </c>
+      <c r="K136" t="n">
+        <v>46</v>
+      </c>
+      <c r="L136" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="M136" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="N136" t="n">
+        <v>-4.6</v>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P136" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>7</v>
+      </c>
+      <c r="C137" t="n">
+        <v>6</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F137" t="n">
+        <v>6</v>
+      </c>
+      <c r="G137" t="n">
+        <v>0</v>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Big Bard</t>
+        </is>
+      </c>
+      <c r="I137" t="n">
+        <v>8</v>
+      </c>
+      <c r="J137" t="n">
+        <v>135</v>
+      </c>
+      <c r="K137" t="n">
+        <v>60</v>
+      </c>
+      <c r="L137" t="inlineStr"/>
+      <c r="M137" t="n">
+        <v>73.28</v>
+      </c>
+      <c r="N137" t="inlineStr"/>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P137" t="n">
+        <v>-11.5</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>7</v>
+      </c>
+      <c r="C138" t="n">
+        <v>6</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F138" t="n">
+        <v>6</v>
+      </c>
+      <c r="G138" t="n">
+        <v>1</v>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Dancing With Drums (IRE)</t>
+        </is>
+      </c>
+      <c r="I138" t="n">
+        <v>4</v>
+      </c>
+      <c r="J138" t="n">
+        <v>131</v>
+      </c>
+      <c r="K138" t="n">
+        <v>56</v>
+      </c>
+      <c r="L138" t="inlineStr"/>
+      <c r="M138" t="n">
+        <v>73.28</v>
+      </c>
+      <c r="N138" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P138" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>7</v>
+      </c>
+      <c r="C139" t="n">
+        <v>6</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F139" t="n">
+        <v>6</v>
+      </c>
+      <c r="G139" t="n">
+        <v>2</v>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Hint Of The Jungle (IRE)</t>
+        </is>
+      </c>
+      <c r="I139" t="n">
+        <v>5</v>
+      </c>
+      <c r="J139" t="n">
+        <v>135</v>
+      </c>
+      <c r="K139" t="n">
+        <v>60</v>
+      </c>
+      <c r="L139" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="M139" t="n">
+        <v>73.28</v>
+      </c>
+      <c r="N139" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P139" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>7</v>
+      </c>
+      <c r="C140" t="n">
+        <v>6</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F140" t="n">
+        <v>6</v>
+      </c>
+      <c r="G140" t="n">
+        <v>3</v>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Elvetham (IRE)</t>
+        </is>
+      </c>
+      <c r="I140" t="n">
+        <v>4</v>
+      </c>
+      <c r="J140" t="n">
+        <v>135</v>
+      </c>
+      <c r="K140" t="n">
+        <v>60</v>
+      </c>
+      <c r="L140" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="M140" t="n">
+        <v>73.28</v>
+      </c>
+      <c r="N140" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P140" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>7</v>
+      </c>
+      <c r="C141" t="n">
+        <v>6</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F141" t="n">
+        <v>6</v>
+      </c>
+      <c r="G141" t="n">
+        <v>4</v>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Rye</t>
+        </is>
+      </c>
+      <c r="I141" t="n">
+        <v>4</v>
+      </c>
+      <c r="J141" t="n">
+        <v>134</v>
+      </c>
+      <c r="K141" t="n">
+        <v>59</v>
+      </c>
+      <c r="L141" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="M141" t="n">
+        <v>73.28</v>
+      </c>
+      <c r="N141" t="n">
+        <v>54</v>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P141" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>7</v>
+      </c>
+      <c r="C142" t="n">
+        <v>6</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F142" t="n">
+        <v>6</v>
+      </c>
+      <c r="G142" t="n">
+        <v>5</v>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Respectable Jack</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>5</v>
+      </c>
+      <c r="J142" t="n">
+        <v>129</v>
+      </c>
+      <c r="K142" t="n">
+        <v>54</v>
+      </c>
+      <c r="L142" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="M142" t="n">
+        <v>73.28</v>
+      </c>
+      <c r="N142" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P142" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>7</v>
+      </c>
+      <c r="C143" t="n">
+        <v>6</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F143" t="n">
+        <v>6</v>
+      </c>
+      <c r="G143" t="n">
+        <v>6</v>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>6</v>
+      </c>
+      <c r="J143" t="n">
+        <v>132</v>
+      </c>
+      <c r="K143" t="n">
+        <v>57</v>
+      </c>
+      <c r="L143" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="M143" t="n">
+        <v>73.28</v>
+      </c>
+      <c r="N143" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P143" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>7</v>
+      </c>
+      <c r="C144" t="n">
+        <v>6</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F144" t="n">
+        <v>6</v>
+      </c>
+      <c r="G144" t="n">
+        <v>7</v>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Court Of Session</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>7</v>
+      </c>
+      <c r="J144" t="n">
+        <v>132</v>
+      </c>
+      <c r="K144" t="n">
+        <v>57</v>
+      </c>
+      <c r="L144" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="M144" t="n">
+        <v>73.28</v>
+      </c>
+      <c r="N144" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P144" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>7</v>
+      </c>
+      <c r="C145" t="n">
+        <v>6</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F145" t="n">
+        <v>6</v>
+      </c>
+      <c r="G145" t="n">
+        <v>8</v>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Unico</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>5</v>
+      </c>
+      <c r="J145" t="n">
+        <v>133</v>
+      </c>
+      <c r="K145" t="n">
+        <v>58</v>
+      </c>
+      <c r="L145" t="n">
+        <v>7.35</v>
+      </c>
+      <c r="M145" t="n">
+        <v>73.28</v>
+      </c>
+      <c r="N145" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P145" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>7</v>
+      </c>
+      <c r="C146" t="n">
+        <v>6</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F146" t="n">
+        <v>6</v>
+      </c>
+      <c r="G146" t="n">
+        <v>9</v>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Man On A Mission</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>7</v>
+      </c>
+      <c r="J146" t="n">
+        <v>132</v>
+      </c>
+      <c r="K146" t="n">
+        <v>57</v>
+      </c>
+      <c r="L146" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="M146" t="n">
+        <v>73.28</v>
+      </c>
+      <c r="N146" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P146" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>7</v>
+      </c>
+      <c r="C147" t="n">
+        <v>6</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F147" t="n">
+        <v>6</v>
+      </c>
+      <c r="G147" t="n">
+        <v>10</v>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Lethal Blast</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>9</v>
+      </c>
+      <c r="J147" t="n">
+        <v>130</v>
+      </c>
+      <c r="K147" t="n">
+        <v>55</v>
+      </c>
+      <c r="L147" t="n">
+        <v>12.35</v>
+      </c>
+      <c r="M147" t="n">
+        <v>73.28</v>
+      </c>
+      <c r="N147" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P147" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>KEMPTON PARK</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>7</v>
+      </c>
+      <c r="C148" t="n">
+        <v>6</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Standard To Slow</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>All Weather</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>6</v>
+      </c>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Fletchers Flight (IRE)</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>6</v>
+      </c>
+      <c r="J148" t="n">
+        <v>134</v>
+      </c>
+      <c r="K148" t="n">
+        <v>59</v>
+      </c>
+      <c r="L148" t="inlineStr"/>
+      <c r="M148" t="n">
+        <v>73.28</v>
+      </c>
+      <c r="N148" t="inlineStr"/>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>